<commit_message>
Re-worked some things to be able to publish now linked to https://global-health-data.org/HealthSystemIndicators/
</commit_message>
<xml_diff>
--- a/RSSH-profile-dash/data/URLs.xlsx
+++ b/RSSH-profile-dash/data/URLs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tommeijer/Git/RSSH-profile-dash/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD738839-12E3-A24A-9FC8-0B0B0D3EB215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08659AAE-DE5B-3440-8FF6-9A0684A5C638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21600" xr2:uid="{4D229E5C-7F44-1549-8816-9B092FBF092C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
   <si>
     <t>Indicator</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Maternal Mortality Rate (MMR)</t>
   </si>
   <si>
-    <t>Coverage of immunisation of children (DTP3)</t>
-  </si>
-  <si>
     <t>Medical Doctors (per 10k pop)</t>
   </si>
   <si>
@@ -86,9 +83,6 @@
     <t>https://www.unfpa.org/sites/default/files/pub-pdf/9789240108462-eng.pdf</t>
   </si>
   <si>
-    <t>https://www.who.int/data/gho/data/indicators/indicator-details/GHO/diphtheria-tetanus-toxoid-and-pertussis-(dtp3)-immunization-coverage-among-1-year-olds-(-)</t>
-  </si>
-  <si>
     <t>https://www.who.int/data/gho/data/indicators/indicator-details/GHO/out-of-pocket-expenditure-(oop)-per-capita-in-us</t>
   </si>
   <si>
@@ -123,6 +117,27 @@
   </si>
   <si>
     <t>UNFPA</t>
+  </si>
+  <si>
+    <t>Coverage of immunisation of children (DTP1)</t>
+  </si>
+  <si>
+    <t>WUENIC</t>
+  </si>
+  <si>
+    <t>https://immunizationdata.who.int/global/wiise-detail-page/diphtheria-tetanus-toxoid-and-pertussis-(dtp)-vaccination-coverage?GROUP=Countries&amp;ANTIGEN=DTPCV1&amp;YEAR=&amp;CODE=</t>
+  </si>
+  <si>
+    <t>DTP1_equity</t>
+  </si>
+  <si>
+    <t>ANC4_equity</t>
+  </si>
+  <si>
+    <t>https://www.countdown2030.org/equity-profiles</t>
+  </si>
+  <si>
+    <t>Countdown to 2030</t>
   </si>
 </sst>
 </file>
@@ -503,12 +518,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A8F8E3E-F66D-A547-BAF4-75BFACB48EEB}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="41.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="141.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="147.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -516,7 +531,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -527,7 +542,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
@@ -538,10 +553,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -549,10 +564,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -560,76 +575,76 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -637,21 +652,43 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
         <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -660,14 +697,15 @@
     <hyperlink ref="C4" r:id="rId2" xr:uid="{6F4EEB9E-4583-724E-844D-FBBBCF992AF7}"/>
     <hyperlink ref="C3" r:id="rId3" xr:uid="{3F488CE1-AD04-9B41-9EA5-90A9CA423437}"/>
     <hyperlink ref="C5" r:id="rId4" xr:uid="{BC5DA9F3-3B0E-5F4D-91A7-7028A5F88471}"/>
-    <hyperlink ref="C6" r:id="rId5" xr:uid="{5F864665-9700-CF46-8FE1-666210926B1B}"/>
-    <hyperlink ref="C7" r:id="rId6" xr:uid="{9F31D254-3661-4B4E-803A-36744B426DE3}"/>
-    <hyperlink ref="C13" r:id="rId7" xr:uid="{E09DA3EF-3AB2-FC4D-9B13-20A518A4179A}"/>
-    <hyperlink ref="C8" r:id="rId8" xr:uid="{8FA3DADC-9870-4845-B98D-ADCC1C4AB84E}"/>
-    <hyperlink ref="C9" r:id="rId9" xr:uid="{17E6CD54-8CA2-A345-8295-88A2FEA740FF}"/>
-    <hyperlink ref="C10" r:id="rId10" xr:uid="{C8286E76-5741-A94E-A50A-108CCB0599D9}"/>
-    <hyperlink ref="C11" r:id="rId11" xr:uid="{9A5BAD2C-D66E-6F47-BE31-120FCE701FDB}"/>
-    <hyperlink ref="C12" r:id="rId12" xr:uid="{578BB956-5256-6042-AA03-2F57927A17ED}"/>
+    <hyperlink ref="C7" r:id="rId5" xr:uid="{5F864665-9700-CF46-8FE1-666210926B1B}"/>
+    <hyperlink ref="C15" r:id="rId6" xr:uid="{E09DA3EF-3AB2-FC4D-9B13-20A518A4179A}"/>
+    <hyperlink ref="C10" r:id="rId7" xr:uid="{8FA3DADC-9870-4845-B98D-ADCC1C4AB84E}"/>
+    <hyperlink ref="C11" r:id="rId8" xr:uid="{17E6CD54-8CA2-A345-8295-88A2FEA740FF}"/>
+    <hyperlink ref="C12" r:id="rId9" xr:uid="{C8286E76-5741-A94E-A50A-108CCB0599D9}"/>
+    <hyperlink ref="C13" r:id="rId10" xr:uid="{9A5BAD2C-D66E-6F47-BE31-120FCE701FDB}"/>
+    <hyperlink ref="C14" r:id="rId11" xr:uid="{578BB956-5256-6042-AA03-2F57927A17ED}"/>
+    <hyperlink ref="C6" r:id="rId12" xr:uid="{F2D73345-673D-974D-9D05-CDEF7757E7E2}"/>
+    <hyperlink ref="C9" r:id="rId13" xr:uid="{EB9A43AA-CF92-EB41-8FA7-FBFBC116EAFB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>